<commit_message>
Add keep_compatible support to MAIN in input excel, adjust docs to deploy with (pre)releases
</commit_message>
<xml_diff>
--- a/examples/excel/example_input_excel.xlsx
+++ b/examples/excel/example_input_excel.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louisparkes-talbot/Desktop/local_model/pyetm/examples/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3D3B6C-2999-CA44-8BC0-89E2ADC9BAC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB6277B2-840B-9948-B6E4-BCD9528A7041}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{AF0205CE-FE76-0D48-9891-27D9A9214571}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>title</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>nl2023</t>
+  </si>
+  <si>
+    <t>keep_compatible</t>
   </si>
 </sst>
 </file>
@@ -596,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA1CC4F3-E0C5-A348-8436-C05118654EF6}">
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
@@ -604,22 +607,23 @@
     <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.1640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.1640625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>4</v>
       </c>
@@ -636,22 +640,25 @@
         <v>0</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
         <v>16</v>
       </c>
@@ -659,17 +666,18 @@
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="7"/>
+      <c r="G2" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G2" s="5">
+      <c r="H2" s="5">
         <v>2050</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="7"/>
+      <c r="I2" s="5"/>
       <c r="J2" s="7"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K2" s="7"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
@@ -677,23 +685,25 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="5"/>
       <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="8"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="5"/>
+      <c r="F4" s="7"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="7"/>
@@ -701,95 +711,103 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="5"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H5" s="7"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="5"/>
+      <c r="F6" s="7"/>
       <c r="G6" s="5"/>
       <c r="H6" s="5"/>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K6" s="5"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
-      <c r="F7" s="5"/>
+      <c r="F7" s="7"/>
       <c r="G7" s="5"/>
       <c r="H7" s="5"/>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
-      <c r="F8" s="5"/>
+      <c r="F8" s="7"/>
       <c r="G8" s="5"/>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K8" s="5"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
-      <c r="F9" s="5"/>
+      <c r="F9" s="7"/>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
-      <c r="F10" s="5"/>
+      <c r="F10" s="7"/>
       <c r="G10" s="5"/>
       <c r="H10" s="5"/>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="5"/>
+      <c r="F11" s="7"/>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
-      <c r="F12" s="5"/>
+      <c r="F12" s="7"/>
       <c r="G12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K12" s="5"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -800,441 +818,478 @@
       <c r="H13" s="5"/>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13" s="5"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
-      <c r="F14" s="5"/>
+      <c r="F14" s="7"/>
       <c r="G14" s="5"/>
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
-      <c r="F15" s="5"/>
+      <c r="F15" s="7"/>
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
-      <c r="F16" s="5"/>
+      <c r="F16" s="7"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K16" s="5"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
-      <c r="F17" s="5"/>
+      <c r="F17" s="7"/>
       <c r="G17" s="5"/>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K17" s="5"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
-      <c r="F18" s="5"/>
+      <c r="F18" s="7"/>
       <c r="G18" s="5"/>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
-      <c r="F19" s="5"/>
+      <c r="F19" s="7"/>
       <c r="G19" s="5"/>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
-      <c r="F20" s="5"/>
+      <c r="F20" s="7"/>
       <c r="G20" s="5"/>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="5"/>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
       <c r="D21" s="5"/>
       <c r="E21" s="7"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="5"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="7"/>
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="5"/>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
       <c r="D22" s="5"/>
       <c r="E22" s="7"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="5"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="7"/>
       <c r="I22" s="5"/>
       <c r="J22" s="5"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
       <c r="D23" s="5"/>
       <c r="E23" s="7"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="5"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="7"/>
       <c r="I23" s="5"/>
       <c r="J23" s="5"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="5"/>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
       <c r="D24" s="5"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="5"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="7"/>
       <c r="I24" s="5"/>
       <c r="J24" s="5"/>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="5"/>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="7"/>
-      <c r="F25" s="5"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="5"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="7"/>
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="5"/>
       <c r="B26" s="5"/>
       <c r="C26" s="5"/>
       <c r="D26" s="5"/>
       <c r="E26" s="7"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="5"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="7"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="5"/>
       <c r="C27" s="5"/>
       <c r="D27" s="5"/>
       <c r="E27" s="7"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="7"/>
-      <c r="H27" s="5"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="7"/>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K27" s="5"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
       <c r="B28" s="5"/>
       <c r="C28" s="5"/>
       <c r="D28" s="5"/>
       <c r="E28" s="7"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="5"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="7"/>
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K28" s="5"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="5"/>
       <c r="E29" s="7"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="5"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="7"/>
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K29" s="5"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>
       <c r="B30" s="5"/>
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="5"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="7"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="5"/>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="7"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="5"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="7"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="5"/>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
       <c r="D32" s="5"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="7"/>
-      <c r="H32" s="5"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="7"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="5"/>
       <c r="B33" s="5"/>
       <c r="C33" s="5"/>
       <c r="D33" s="5"/>
       <c r="E33" s="7"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="7"/>
-      <c r="H33" s="5"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="7"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="5"/>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
       <c r="D34" s="5"/>
       <c r="E34" s="7"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="5"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="7"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="5"/>
       <c r="B35" s="5"/>
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="7"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="7"/>
-      <c r="H35" s="5"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="5"/>
+      <c r="H35" s="7"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="5"/>
       <c r="B36" s="5"/>
       <c r="C36" s="5"/>
       <c r="D36" s="5"/>
       <c r="E36" s="7"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="7"/>
-      <c r="H36" s="5"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="7"/>
       <c r="I36" s="5"/>
       <c r="J36" s="5"/>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" s="5"/>
       <c r="B37" s="5"/>
       <c r="C37" s="5"/>
       <c r="D37" s="5"/>
       <c r="E37" s="7"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="7"/>
-      <c r="H37" s="5"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="7"/>
       <c r="I37" s="5"/>
       <c r="J37" s="5"/>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="5"/>
       <c r="D38" s="5"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="5"/>
-      <c r="G38" s="7"/>
-      <c r="H38" s="5"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="7"/>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="5"/>
       <c r="B39" s="5"/>
       <c r="C39" s="5"/>
       <c r="D39" s="5"/>
       <c r="E39" s="7"/>
-      <c r="F39" s="5"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="5"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="5"/>
+      <c r="H39" s="7"/>
       <c r="I39" s="5"/>
       <c r="J39" s="5"/>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" s="5"/>
       <c r="B40" s="5"/>
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="7"/>
-      <c r="F40" s="5"/>
-      <c r="G40" s="7"/>
-      <c r="H40" s="5"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="7"/>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K40" s="5"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="5"/>
       <c r="B41" s="5"/>
       <c r="C41" s="5"/>
       <c r="D41" s="5"/>
       <c r="E41" s="7"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="5"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="7"/>
       <c r="I41" s="5"/>
       <c r="J41" s="5"/>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="5"/>
       <c r="D42" s="5"/>
       <c r="E42" s="7"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="7"/>
-      <c r="H42" s="5"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="7"/>
       <c r="I42" s="5"/>
       <c r="J42" s="5"/>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" s="5"/>
       <c r="B43" s="5"/>
       <c r="C43" s="5"/>
       <c r="D43" s="5"/>
       <c r="E43" s="7"/>
-      <c r="F43" s="5"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="5"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="7"/>
       <c r="I43" s="5"/>
       <c r="J43" s="5"/>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" s="5"/>
       <c r="B44" s="5"/>
       <c r="C44" s="5"/>
       <c r="D44" s="5"/>
       <c r="E44" s="7"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="7"/>
-      <c r="H44" s="5"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="7"/>
       <c r="I44" s="5"/>
       <c r="J44" s="5"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K44" s="5"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" s="5"/>
       <c r="B45" s="5"/>
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="7"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="5"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="5"/>
+      <c r="H45" s="7"/>
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" s="5"/>
       <c r="B46" s="5"/>
       <c r="C46" s="5"/>
       <c r="D46" s="5"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="7"/>
-      <c r="H46" s="5"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="7"/>
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K46" s="5"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" s="5"/>
       <c r="B47" s="5"/>
       <c r="C47" s="5"/>
       <c r="D47" s="5"/>
       <c r="E47" s="7"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="5"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="5"/>
+      <c r="H47" s="7"/>
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" s="5"/>
       <c r="B48" s="5"/>
       <c r="C48" s="5"/>
       <c r="D48" s="5"/>
       <c r="E48" s="7"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="7"/>
-      <c r="H48" s="5"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="5"/>
+      <c r="H48" s="7"/>
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K48" s="5"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" s="5"/>
       <c r="B49" s="5"/>
       <c r="C49" s="5"/>
       <c r="D49" s="5"/>
       <c r="E49" s="7"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="7"/>
-      <c r="H49" s="5"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="5"/>
+      <c r="H49" s="7"/>
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A3 D2:J3 B4:J4 C5:J12 C14:E20 F14:J49 A21:E49">
+  <conditionalFormatting sqref="A2:A3 D2:K3 B4:K4 C5:K12 C14:F20 G14:K49 A21:F49">
     <cfRule type="notContainsBlanks" dxfId="5" priority="31">
       <formula>LEN(TRIM(A2))&gt;0</formula>
     </cfRule>

</xml_diff>